<commit_message>
feat: update Milvus few-shot store with new vector data and improve RAG retrieval filtering logic
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,6 +461,155 @@
           <t>Error</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-30 18:19:39</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>bba7deed-8409-4338-87c3-f40338fda613</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>which schools in eluru have the highest number of dropouts in 2025</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SELECT d.district_name, COUNT(*) as dropout_count FROM ap_citizen360.dim_student s JOIN ap_citizen360.dim_district d ON s.institution_code = d.district_id WHERE s.is_dropout = 1 AND s.academic_year IN ('2025', '2024') GROUP BY d.district_name ORDER BY dropout_count DESC</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>The query ran successfully but returned no rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-30 18:24:22</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>6c0bf5cd-f050-45cd-9f53-d209f923f95c</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>which schools in eluru have the highest number of dropouts in 2025</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SELECT d.district_name, COUNT(*) as dropout_count FROM ap_citizen360.dim_student s JOIN ap_citizen360.dim_district d ON s.institution_code = d.district_id WHERE s.academic_year IN ('2025', '2024') GROUP BY d.district_name ORDER BY dropout_count DESC</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>The query ran successfully but returned no rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-30 18:26:16</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>428fbf28-e0f0-4796-9c5a-40e030a7d341</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>which schools in eluru have the highest number of dropouts in 2025</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SELECT d.district_name, COUNT(*) as dropout_count FROM ap_citizen360_dim_student s JOIN ap_citizen360_dim_district d ON s.institution_code = d.district_id WHERE s.academic_year IN ('2025', '2024') GROUP BY d.district_name ORDER BY dropout_count DESC</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>The query ran successfully but returned no rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-30 18:29:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ab817bb7-6703-48a6-a87d-1d253993b86b</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>which schools in eluru have the highest number of dropouts in 2025</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SELECT s.school_name, COUNT(s.student_record_id) AS dropout_count FROM dim_student s JOIN dim_facility_school f ON s.institution_id = f.canonical_facility_id WHERE s.academic_year = '2025' AND s.is_dropout = TRUE GROUP BY s.school_name ORDER BY dropout_count DESC</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>The query ran successfully but returned no rows.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
refactor: remove legacy facility schema definitions and update associated RAG pipeline configurations
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -609,7 +609,539 @@
           <t>The query ran successfully but returned no rows.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:01:45</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>f580a567-e207-4806-83f4-61ec9d68cb8f</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>How many students dropped out in 2025-26?</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>cancelled</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Request cancelled by user.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:04:23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>perf_test_1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>How many students dropped out in 2025-26?</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>To answer your question about how many students dropped out in 2025-26, I need to use the available tools to retrieve the actual data from the database.
+First, let me get the schema details to confirm the table names and columns:</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>To answer your question about how many students dropped out in 2025-26, I need to use the available tools to retrieve the actual data from the database.
+First, let me get the schema details to confirm the table names and columns:</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:05:02</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>perf_test_2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>List the top 5 districts with the highest dropout count.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>model 'qwen3.5:0.8b-mlx' not found (status code: 404)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:06:37</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>perf_test_1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>How many students dropped out in 2025-26?</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SELECT COUNT(*) AS dropout_count FROM dim_student WHERE academic_year = '2025-26' AND is_dropout = TRUE</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>**0** (dropout count).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:10:05</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>perf_test_2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>List the top 5 districts with the highest dropout count.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SELECT district_name, COUNT(*) AS dropout_count FROM fact_benefit_transaction JOIN dim_person ON fact_benefit_transaction.person_id = dim_person.person_id WHERE fact_benefit_transaction.district_id = dim_district.district_id AND dim_student.is_dropout = TRUE GROUP BY district_name ORDER BY dropout_count DESC LIMIT 5</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SQL execution failed: (sqlite3.OperationalError) no such column: district_name
+[SQL: SELECT district_name, COUNT(*) AS dropout_count FROM fact_benefit_transaction JOIN dim_person ON fact_benefit_transaction.person_id = dim_person.person_id WHERE fact_benefit_transaction.district_id = dim_district.district_id AND dim_student.is_dropout = TRUE GROUP BY district_name ORDER BY dropout_count DESC LIMIT 5]
+(Background on this error at: https://sqlalche.me/e/20/e3q8)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>(sqlite3.OperationalError) no such column: district_name
+[SQL: SELECT district_name, COUNT(*) AS dropout_count FROM fact_benefit_transaction JOIN dim_person ON fact_benefit_transaction.person_id = dim_person.person_id WHERE fact_benefit_transaction.district_id = dim_district.district_id AND dim_student.is_dropout = TRUE GROUP BY district_name ORDER BY dropout_count DESC LIMIT 5]
+(Background on this error at: https://sqlalche.me/e/20/e3q8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:13:23</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>perf_test_3</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>What is the gender distribution of dropouts?</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SELECT gender, COUNT(*) AS dropout_count FROM dim_student WHERE is_dropout = TRUE AND gender = 'Female' GROUP BY gender ORDER BY dropout_count DESC</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>SQL execution failed: (sqlite3.OperationalError) no such column: gender
+[SQL: SELECT gender, COUNT(*) AS dropout_count FROM dim_student WHERE is_dropout = TRUE AND gender = 'Female' GROUP BY gender ORDER BY dropout_count DESC]
+(Background on this error at: https://sqlalche.me/e/20/e3q8)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>(sqlite3.OperationalError) no such column: gender
+[SQL: SELECT gender, COUNT(*) AS dropout_count FROM dim_student WHERE is_dropout = TRUE AND gender = 'Female' GROUP BY gender ORDER BY dropout_count DESC]
+(Background on this error at: https://sqlalche.me/e/20/e3q8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:15:19</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>perf_test_4</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Show me dropout reasons and their counts.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>model 'qwen3.5:2b-mlx' not found (status code: 404)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:16:27</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>perf_test_1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>How many students dropped out in 2025-26?</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SELECT COUNT(*) AS dropout_count FROM dim_student s JOIN dim_person p ON s.person_id = p.person_id JOIN dim_district d ON p.district_id = d.district_id WHERE s.academic_year = '2025-26' AND s.is_dropout = TRUE AND d.district_name = 'ANANTHAPURAMU'</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>**0** (dropout count).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:18:06</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>perf_test_2</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>List the top 5 districts with the highest dropout count.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>SELECT district_name, COUNT(*) AS dropout_count FROM fact_benefit_transaction JOIN dim_person ON fact_benefit_transaction.person_id = dim_person.person_id WHERE fact_benefit_transaction.district_id = dim_district.district_id AND dim_student.is_dropout = TRUE GROUP BY district_name ORDER BY dropout_count DESC LIMIT 5</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>SQL execution failed: (sqlite3.OperationalError) no such column: district_name
+[SQL: SELECT district_name, COUNT(*) AS dropout_count FROM fact_benefit_transaction JOIN dim_person ON fact_benefit_transaction.person_id = dim_person.person_id WHERE fact_benefit_transaction.district_id = dim_district.district_id AND dim_student.is_dropout = TRUE GROUP BY district_name ORDER BY dropout_count DESC LIMIT 5]
+(Background on this error at: https://sqlalche.me/e/20/e3q8)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>(sqlite3.OperationalError) no such column: district_name
+[SQL: SELECT district_name, COUNT(*) AS dropout_count FROM fact_benefit_transaction JOIN dim_person ON fact_benefit_transaction.person_id = dim_person.person_id WHERE fact_benefit_transaction.district_id = dim_district.district_id AND dim_student.is_dropout = TRUE GROUP BY district_name ORDER BY dropout_count DESC LIMIT 5]
+(Background on this error at: https://sqlalche.me/e/20/e3q8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:19:38</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>perf_test_3</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>What is the gender distribution of dropouts?</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>SELECT gender, COUNT(*) AS dropout_count FROM dim_student WHERE is_dropout = TRUE AND gender = 'Female' GROUP BY gender ORDER BY dropout_count DESC</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>SQL execution failed: (sqlite3.OperationalError) no such column: gender
+[SQL: SELECT gender, COUNT(*) AS dropout_count FROM dim_student WHERE is_dropout = TRUE AND gender = 'Female' GROUP BY gender ORDER BY dropout_count DESC]
+(Background on this error at: https://sqlalche.me/e/20/e3q8)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>(sqlite3.OperationalError) no such column: gender
+[SQL: SELECT gender, COUNT(*) AS dropout_count FROM dim_student WHERE is_dropout = TRUE AND gender = 'Female' GROUP BY gender ORDER BY dropout_count DESC]
+(Background on this error at: https://sqlalche.me/e/20/e3q8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:22:05</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>perf_test_4</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Show me dropout reasons and their counts.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SELECT 
+    s.student_record_id,
+    p.person_name,
+    d.district_id,
+    m.mandal_id,
+    v.village_name,
+    h.household_id,
+    h.household_income_category,
+    h.village_name,
+    h.land_type,
+    h.household_count,
+    s.is_dropout,
+    s.dropout_reason,
+    COUNT(*) as dropout_count
+FROM dim_student s
+JOIN dim_person p ON s.person_id = p.person_id
+JOIN dim_household h ON p.household_id = h.household_id
+WHERE s.is_dropout = TRUE
+GROUP BY s.student_record_id, p.person_name, d.district_id, m.mandal_id, v.village_name, h.household_id, h.household_income_category, h.village_name, h.land_type, h.household_count</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>SQL execution failed: (sqlite3.OperationalError) no such column: d.district_id
+[SQL: SELECT 
+    s.student_record_id,
+    p.person_name,
+    d.district_id,
+    m.mandal_id,
+    v.village_name,
+    h.household_id,
+    h.household_income_category,
+    h.village_name,
+    h.land_type,
+    h.household_count,
+    s.is_dropout,
+    s.dropout_reason,
+    COUNT(*) as dropout_count
+FROM dim_student s
+JOIN dim_person p ON s.person_id = p.person_id
+JOIN dim_household h ON p.household_id = h.household_id
+WHERE s.is_dropout = TRUE
+GROUP BY s.student_record_id, p.person_name, d.district_id, m.mandal_id, v.village_name, h.household_id, h.household_income_category, h.village_name, h.land_type, h.household_count]
+(Background on this error at: https://sqlalche.me/e/20/e3q8)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>(sqlite3.OperationalError) no such column: d.district_id
+[SQL: SELECT 
+    s.student_record_id,
+    p.person_name,
+    d.district_id,
+    m.mandal_id,
+    v.village_name,
+    h.household_id,
+    h.household_income_category,
+    h.village_name,
+    h.land_type,
+    h.household_count,
+    s.is_dropout,
+    s.dropout_reason,
+    COUNT(*) as dropout_count
+FROM dim_student s
+JOIN dim_person p ON s.person_id = p.person_id
+JOIN dim_household h ON p.household_id = h.household_id
+WHERE s.is_dropout = TRUE
+GROUP BY s.student_record_id, p.person_name, d.district_id, m.mandal_id, v.village_name, h.household_id, h.household_income_category, h.village_name, h.land_type, h.household_count]
+(Background on this error at: https://sqlalche.me/e/20/e3q8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:24:15</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>perf_test_5</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>How many SC category students dropped out in Anantapur?</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>To answer your question about how many SC category students dropped out in Anantapur, I need to use the available tools to retrieve the actual data from the database.
+First, let me get the schema details to confirm the table names and columns:</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>To answer your question about how many SC category students dropped out in Anantapur, I need to use the available tools to retrieve the actual data from the database.
+First, let me get the schema details to confirm the table names and columns:</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: add latency tracking columns for generation, execution, and total time to query log
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,21 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Error</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Gen Time (s)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Exec Time (s)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Total Time (s)</t>
         </is>
       </c>
     </row>
@@ -2192,6 +2207,53 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-05 11:19:29</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>test_session</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>what is the count?</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SELECT COUNT(*) FROM table</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Count is 10</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="K45" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: resolve ClosedResourceError in MCP tool execution by stabilizing session management in app.py and mcp_rag.py
</commit_message>
<xml_diff>
--- a/ap_citizen360_v1.5.2/database/query_log.xlsx
+++ b/ap_citizen360_v1.5.2/database/query_log.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2243,7 +2243,6 @@
           <t>Count is 10</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
       <c r="I45" t="n">
         <v>2.1</v>
       </c>
@@ -2252,6 +2251,198 @@
       </c>
       <c r="K45" t="n">
         <v>2.5</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-19 19:36:48</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>prakhars</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>78431676-fee9-4002-a49d-f43285a7722a</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>show 5 schools in guntur</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>3.86</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-19 19:41:44</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>prakhars</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>78431676-fee9-4002-a49d-f43285a7722a</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>show 5 schools in guntur</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-19 19:52:38</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>9e184090-98dd-44c3-9d0f-37c5b9d0c81b</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>total students</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>3.78</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-19 19:57:06</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>e4e2a6a2-eb47-4e6f-ba6d-10ed9b7051eb</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>show 5 schools in guntur</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>cancelled</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Request cancelled by user.</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="n">
+        <v>28.88</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-19 19:58:12</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>test_user</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>e4e2a6a2-eb47-4e6f-ba6d-10ed9b7051eb</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>show 5 schools in guntur</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Empty query</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>50.51</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="K50" t="n">
+        <v>52.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>